<commit_message>
Test suggested fixes with near-miss sample rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Fixtures/imports/clients.xlsx
+++ b/tests/Fixtures/imports/clients.xlsx
@@ -68,7 +68,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M21"/>
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="0" t="inlineStr">
@@ -890,6 +890,239 @@
       <c r="M16" s="0" t="inlineStr">
         <is>
           <t>Month written out</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Nina Cruz</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>0917 222 8888</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>nina.cruz@example.com</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>25/12/1988</t>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t>Marikina</t>
+        </is>
+      </c>
+      <c r="M17" s="0" t="inlineStr">
+        <is>
+          <t>Day-first birthday</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Ben Torres</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>0918 333 4444</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>ben.torres@gmial.com</t>
+        </is>
+      </c>
+      <c r="D18" s="1">
+        <v>30378</v>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>Married</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t>Antipolo</t>
+        </is>
+      </c>
+      <c r="M18" s="0" t="inlineStr">
+        <is>
+          <t>Email domain typo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>Carmen Ong</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>0919 444 5555</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>carmen.ong@example.com</t>
+        </is>
+      </c>
+      <c r="D19" s="1">
+        <v>29043</v>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>Married</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>San Juan</t>
+        </is>
+      </c>
+      <c r="G19" s="0" t="inlineStr">
+        <is>
+          <t>Health Shield</t>
+        </is>
+      </c>
+      <c r="H19" s="0" t="inlineStr">
+        <is>
+          <t>HS-20010</t>
+        </is>
+      </c>
+      <c r="I19" s="0" t="inlineStr">
+        <is>
+          <t>1,800</t>
+        </is>
+      </c>
+      <c r="J19" s="0" t="inlineStr">
+        <is>
+          <t>Monthy</t>
+        </is>
+      </c>
+      <c r="K19" s="1">
+        <v>45717</v>
+      </c>
+      <c r="L19" s="0" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M19" s="0" t="inlineStr">
+        <is>
+          <t>Payment mode typo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Dan Ramos</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>0917 765 4321 (home)</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>dan.ramos@example.com</t>
+        </is>
+      </c>
+      <c r="D20" s="1">
+        <v>31632</v>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>Mandaluyong</t>
+        </is>
+      </c>
+      <c r="M20" s="0" t="inlineStr">
+        <is>
+          <t>Phone with a note</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Elsa Go</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>0920 987 6543</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>elsa.go@example.com</t>
+        </is>
+      </c>
+      <c r="D21" s="1">
+        <v>33553</v>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>Paranaque</t>
+        </is>
+      </c>
+      <c r="G21" s="0" t="inlineStr">
+        <is>
+          <t>Life Plus</t>
+        </is>
+      </c>
+      <c r="H21" s="0" t="inlineStr">
+        <is>
+          <t>LP-10010</t>
+        </is>
+      </c>
+      <c r="I21" s="0" t="inlineStr">
+        <is>
+          <t>₱1,500 per month</t>
+        </is>
+      </c>
+      <c r="J21" s="0" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="K21" s="1">
+        <v>45748</v>
+      </c>
+      <c r="L21" s="0" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M21" s="0" t="inlineStr">
+        <is>
+          <t>Amount with words</t>
         </is>
       </c>
     </row>

</xml_diff>